<commit_message>
Use English throughout the public release and verify data integrity
</commit_message>
<xml_diff>
--- a/04_Figure04/data/source_data/Figure04.xlsx
+++ b/04_Figure04/data/source_data/Figure04.xlsx
@@ -203,8 +203,8 @@
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
         <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Hans" typeface="SimSun"/>
+        <a:font script="Hant" typeface="PMingLiU"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -237,8 +237,8 @@
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
         <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Hans" typeface="SimSun"/>
+        <a:font script="Hant" typeface="PMingLiU"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
         <a:font script="Thai" typeface="Tahoma"/>

</xml_diff>